<commit_message>
Allinea lo script generatore al protocollo da 6 flaconi
Lo script ricostruiva ancora la riga del percorso da 5 (239 euro, 300 mL) e
la voce corrispondente nel foglio Sintesi. Ora coincide con il file .xlsx.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KZs9j8MkWEGcDu1fmJqBFc
</commit_message>
<xml_diff>
--- a/analisi/ricerca/mappa-competitiva.xlsx
+++ b/analisi/ricerca/mappa-competitiva.xlsx
@@ -568,7 +568,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -604,7 +603,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -633,7 +631,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -676,7 +673,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -719,7 +715,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -2777,7 +2772,7 @@
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Nostro costo mensile, percorso da 5</t>
+          <t>Nostro costo mensile, percorso da 6</t>
         </is>
       </c>
       <c r="C12" s="25">

</xml_diff>